<commit_message>
Update Company 1 actual data from latest screenshot
</commit_message>
<xml_diff>
--- a/Oil_Data_Consolidated.xlsx
+++ b/Oil_Data_Consolidated.xlsx
@@ -1542,11 +1542,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>1437030</v>
+      </c>
       <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="inlineStr"/>
+        <v>40000</v>
+      </c>
+      <c r="G44" t="n">
+        <v>16500</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -1567,9 +1571,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>617312</v>
+      </c>
+      <c r="F45" t="n">
+        <v>31000</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -1590,11 +1600,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="n">
+        <v>1318903</v>
+      </c>
       <c r="F46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" t="inlineStr"/>
+        <v>120000</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -1615,9 +1629,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>617312</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -1638,11 +1658,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>1256089</v>
+      </c>
       <c r="F48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" t="inlineStr"/>
+        <v>60000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -1663,9 +1687,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>603447</v>
+      </c>
+      <c r="F49" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -1686,11 +1716,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>1164376</v>
+      </c>
       <c r="F50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" t="inlineStr"/>
+        <v>100000</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -1711,9 +1745,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="E51" t="n">
+        <v>563813</v>
+      </c>
+      <c r="F51" t="n">
+        <v>43000</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -1734,11 +1774,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>1164376</v>
+      </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
-      <c r="G52" t="inlineStr"/>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -1759,9 +1803,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>563284</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -1782,11 +1832,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="n">
+        <v>1164376</v>
+      </c>
       <c r="F54" t="n">
         <v>0</v>
       </c>
-      <c r="G54" t="inlineStr"/>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -1807,9 +1861,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>563284</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -1830,11 +1890,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>998251</v>
+      </c>
       <c r="F56" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" t="inlineStr"/>
+        <v>165830</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -1855,9 +1919,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>524021</v>
+      </c>
+      <c r="F57" t="n">
+        <v>38810</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -1878,11 +1948,15 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>877834</v>
+      </c>
       <c r="F58" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" t="inlineStr"/>
+        <v>120000</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -1903,9 +1977,15 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
+      <c r="E59" t="n">
+        <v>524021</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -1926,11 +2006,13 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>836660</v>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -1951,9 +2033,13 @@
           <t>Petrol</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>491471</v>
+      </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">

</xml_diff>